<commit_message>
Fs theo TT 07/2025 Phụ lục IXa (chì 18.278, pin sạc 54.876 đ/kg); xác minh Chỉ thị 20/CT-TTg; chạy lại business case
</commit_message>
<xml_diff>
--- a/07-business-case/cost-model.xlsx
+++ b/07-business-case/cost-model.xlsx
@@ -580,17 +580,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>18.278 đồng/kg theo bảng định mức Fs (nguồn thứ cấp, chưa thấy văn bản gốc; NĐ 110 Điều 8.2 giao Bộ trưởng ban hành Fs, điều chỉnh lần đầu 2029)</t>
+          <t>18.278 đồng/kg theo TT 07/2025/TT-BTNMT Phụ lục IXa, dòng B.1.1 (SRC-023). Giữ đến 2035; NĐ 110 Điều 8.2 cho điều chỉnh 3 năm/lần từ 2029, max giả định +10%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>H</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>18278</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>22000</t>
+          <t>20106</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fs của pin Li dùng cho phương tiện giao thông khi R &gt; 0 (đồng/kg)</t>
+          <t>Fs của pin Li dùng cho phương tiện giao thông (đồng/kg)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -627,27 +627,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chưa có định mức công bố (R hiện bằng 0%). Giả định cùng bậc với ắc quy chì</t>
+          <t>54.876 đồng/kg theo TT 07/2025/TT-BTNMT Phụ lục IXa, dòng B.2.1 Pin sạc nhiều lần các loại (SRC-023); R hiện bằng 0% nên chưa phát sinh tiền. Min giả định Bộ ban hành mức riêng thấp hơn cho pin phương tiện; max +10% ở lần điều chỉnh 2029</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>25000</t>
+          <t>54876</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>60364</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2199,10 +2199,10 @@
         <v>-743.42</v>
       </c>
       <c r="J25" t="n">
-        <v>1789.34</v>
+        <v>3927.68</v>
       </c>
       <c r="K25" t="n">
-        <v>1342.01</v>
+        <v>2945.76</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -2283,10 +2283,10 @@
         <v>-1183.32</v>
       </c>
       <c r="J27" t="n">
-        <v>2135.6</v>
+        <v>4687.73</v>
       </c>
       <c r="K27" t="n">
-        <v>1601.7</v>
+        <v>3515.8</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -2367,10 +2367,10 @@
         <v>-1767</v>
       </c>
       <c r="J29" t="n">
-        <v>2478.45</v>
+        <v>5440.29</v>
       </c>
       <c r="K29" t="n">
-        <v>1858.84</v>
+        <v>4080.22</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2451,10 +2451,10 @@
         <v>-2492.88</v>
       </c>
       <c r="J31" t="n">
-        <v>5315.57</v>
+        <v>11667.9</v>
       </c>
       <c r="K31" t="n">
-        <v>3986.68</v>
+        <v>8750.92</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2535,10 +2535,10 @@
         <v>-3358.72</v>
       </c>
       <c r="J33" t="n">
-        <v>5993.2</v>
+        <v>13155.31</v>
       </c>
       <c r="K33" t="n">
-        <v>4494.9</v>
+        <v>9866.48</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>-4366.1</v>
       </c>
       <c r="J35" t="n">
-        <v>6674.56</v>
+        <v>14650.94</v>
       </c>
       <c r="K35" t="n">
-        <v>5005.92</v>
+        <v>10988.2</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2703,10 +2703,10 @@
         <v>-5515.41</v>
       </c>
       <c r="J37" t="n">
-        <v>7359.92</v>
+        <v>16155.31</v>
       </c>
       <c r="K37" t="n">
-        <v>5519.94</v>
+        <v>12116.48</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2955,10 +2955,10 @@
         <v>-743.42</v>
       </c>
       <c r="J43" t="n">
-        <v>2236.68</v>
+        <v>4909.6</v>
       </c>
       <c r="K43" t="n">
-        <v>1677.51</v>
+        <v>3682.2</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -3039,10 +3039,10 @@
         <v>-1183.32</v>
       </c>
       <c r="J45" t="n">
-        <v>2669.5</v>
+        <v>5859.66</v>
       </c>
       <c r="K45" t="n">
-        <v>2002.13</v>
+        <v>4394.75</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -3123,10 +3123,10 @@
         <v>-1767</v>
       </c>
       <c r="J47" t="n">
-        <v>3098.06</v>
+        <v>6800.37</v>
       </c>
       <c r="K47" t="n">
-        <v>2323.55</v>
+        <v>5100.28</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -3207,10 +3207,10 @@
         <v>-2492.88</v>
       </c>
       <c r="J49" t="n">
-        <v>7087.43</v>
+        <v>15557.2</v>
       </c>
       <c r="K49" t="n">
-        <v>5315.57</v>
+        <v>11667.9</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -3291,10 +3291,10 @@
         <v>-3358.72</v>
       </c>
       <c r="J51" t="n">
-        <v>7990.93</v>
+        <v>17540.41</v>
       </c>
       <c r="K51" t="n">
-        <v>5993.2</v>
+        <v>13155.31</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -3375,10 +3375,10 @@
         <v>-4366.1</v>
       </c>
       <c r="J53" t="n">
-        <v>8899.42</v>
+        <v>19534.58</v>
       </c>
       <c r="K53" t="n">
-        <v>6674.56</v>
+        <v>14650.94</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -3459,10 +3459,10 @@
         <v>-5515.41</v>
       </c>
       <c r="J55" t="n">
-        <v>9813.219999999999</v>
+        <v>21540.42</v>
       </c>
       <c r="K55" t="n">
-        <v>7359.92</v>
+        <v>16155.31</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -3609,10 +3609,10 @@
         <v>-8279</v>
       </c>
       <c r="D5" t="n">
-        <v>19187</v>
+        <v>41078</v>
       </c>
       <c r="E5" t="n">
-        <v>14607</v>
+        <v>31026</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -3661,10 +3661,10 @@
         <v>-8279</v>
       </c>
       <c r="D7" t="n">
-        <v>24895</v>
+        <v>53607</v>
       </c>
       <c r="E7" t="n">
-        <v>18888</v>
+        <v>40423</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3746,13 +3746,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.898</v>
+        <v>0.991</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.102</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -3830,13 +3830,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.855</v>
+        <v>0.97</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.145</v>
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>
@@ -3922,13 +3922,13 @@
         <v>-4591</v>
       </c>
       <c r="C4" t="n">
-        <v>5819</v>
+        <v>7957</v>
       </c>
       <c r="D4" t="n">
-        <v>10410</v>
+        <v>12548</v>
       </c>
       <c r="E4" t="n">
-        <v>21563</v>
+        <v>23701</v>
       </c>
     </row>
     <row r="5">
@@ -3939,13 +3939,13 @@
         <v>-5735</v>
       </c>
       <c r="C5" t="n">
-        <v>6150</v>
+        <v>8702</v>
       </c>
       <c r="D5" t="n">
-        <v>11885</v>
+        <v>14437</v>
       </c>
       <c r="E5" t="n">
-        <v>33447</v>
+        <v>38138</v>
       </c>
     </row>
     <row r="6">
@@ -3956,13 +3956,13 @@
         <v>-6934</v>
       </c>
       <c r="C6" t="n">
-        <v>6545</v>
+        <v>9507</v>
       </c>
       <c r="D6" t="n">
-        <v>13479</v>
+        <v>16441</v>
       </c>
       <c r="E6" t="n">
-        <v>46926</v>
+        <v>54578</v>
       </c>
     </row>
     <row r="7">
@@ -3973,13 +3973,13 @@
         <v>-8256</v>
       </c>
       <c r="C7" t="n">
-        <v>9406</v>
+        <v>15758</v>
       </c>
       <c r="D7" t="n">
-        <v>17662</v>
+        <v>24015</v>
       </c>
       <c r="E7" t="n">
-        <v>64588</v>
+        <v>78593</v>
       </c>
     </row>
     <row r="8">
@@ -3990,13 +3990,13 @@
         <v>-9706</v>
       </c>
       <c r="C8" t="n">
-        <v>10089</v>
+        <v>17251</v>
       </c>
       <c r="D8" t="n">
-        <v>19795</v>
+        <v>26957</v>
       </c>
       <c r="E8" t="n">
-        <v>84383</v>
+        <v>105550</v>
       </c>
     </row>
     <row r="9">
@@ -4007,13 +4007,13 @@
         <v>-11231</v>
       </c>
       <c r="C9" t="n">
-        <v>10733</v>
+        <v>18709</v>
       </c>
       <c r="D9" t="n">
-        <v>21964</v>
+        <v>29941</v>
       </c>
       <c r="E9" t="n">
-        <v>106347</v>
+        <v>135490</v>
       </c>
     </row>
     <row r="10">
@@ -4024,13 +4024,13 @@
         <v>-12841</v>
       </c>
       <c r="C10" t="n">
-        <v>11351</v>
+        <v>20147</v>
       </c>
       <c r="D10" t="n">
-        <v>24193</v>
+        <v>32988</v>
       </c>
       <c r="E10" t="n">
-        <v>130540</v>
+        <v>168478</v>
       </c>
     </row>
   </sheetData>

</xml_diff>